<commit_message>
in the middle of fixing it all
</commit_message>
<xml_diff>
--- a/test_cases/regcv2_testbench.xlsx
+++ b/test_cases/regcv2_testbench.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="74">
   <si>
     <t>name</t>
   </si>
@@ -51,7 +51,7 @@
     <t>TimeSeries_1</t>
   </si>
   <si>
-    <t>disturbance_profile_15.xlsx</t>
+    <t>disturbance_profile.xlsx</t>
   </si>
   <si>
     <t>PLBVF</t>
@@ -740,7 +740,9 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
+      <c r="B3" s="3" t="s">
+        <v>10</v>
+      </c>
       <c r="C3" s="3"/>
       <c r="D3" s="3"/>
       <c r="E3" s="3"/>
@@ -1247,7 +1249,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:R6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
@@ -1365,6 +1367,7 @@
         <v>0.2</v>
       </c>
     </row>
+    <row r="6" spans="8:8" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>